<commit_message>
Edit warning message and update Power_Parameters.xlsx file
</commit_message>
<xml_diff>
--- a/data/exampleStochastic/Power_Parameters.xlsx
+++ b/data/exampleStochastic/Power_Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo\data\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A658E7-62F7-4FD1-9B9B-EE98D50A0A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC4CDDB-9480-4559-A267-496F079188FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33915" yWindow="-21810" windowWidth="38640" windowHeight="21120" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Parameters" sheetId="121" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
   <si>
     <t>[p.u.]</t>
   </si>
@@ -342,7 +342,13 @@
     <t>Format:</t>
   </si>
   <si>
-    <t>v0.1.0</t>
+    <t>Intra-Day Storage constraint type for edge timesteps</t>
+  </si>
+  <si>
+    <t>pReprPeriodEdgeHandlingIntraDayStorage</t>
+  </si>
+  <si>
+    <t>v0.2.0</t>
   </si>
 </sst>
 </file>
@@ -571,7 +577,21 @@
     <cellStyle name="Standard 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
     <cellStyle name="Standard 4" xfId="7" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="34">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFB90135"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF4E9C49"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1113,7 +1133,7 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="B1:H76"/>
+  <dimension ref="B1:H79"/>
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" style="1" customWidth="1"/>
@@ -1137,7 +1157,7 @@
         <v>91</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1709,16 +1729,46 @@
         <v>71</v>
       </c>
     </row>
+    <row r="78" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B78" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B79" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="C5:C6 C14:C28">
-    <cfRule type="cellIs" dxfId="31" priority="39" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="41" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="42" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8:C9">
+    <cfRule type="cellIs" dxfId="31" priority="101" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="102" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11:C12">
     <cfRule type="cellIs" dxfId="29" priority="99" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1726,23 +1776,23 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11:C12">
-    <cfRule type="cellIs" dxfId="27" priority="97" operator="equal">
+  <conditionalFormatting sqref="C31">
+    <cfRule type="cellIs" dxfId="27" priority="111" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="98" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
-    <cfRule type="cellIs" dxfId="25" priority="109" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="110" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="112" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
+    <cfRule type="cellIs" dxfId="25" priority="89" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="90" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C37 C40">
     <cfRule type="cellIs" dxfId="23" priority="87" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1750,7 +1800,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C37 C40">
+  <conditionalFormatting sqref="C43">
     <cfRule type="cellIs" dxfId="21" priority="85" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1758,7 +1808,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C43">
+  <conditionalFormatting sqref="C46">
     <cfRule type="cellIs" dxfId="19" priority="83" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1766,7 +1816,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C46">
+  <conditionalFormatting sqref="C49">
     <cfRule type="cellIs" dxfId="17" priority="81" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1774,47 +1824,47 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C49">
-    <cfRule type="cellIs" dxfId="15" priority="79" operator="equal">
+  <conditionalFormatting sqref="C53 C56">
+    <cfRule type="cellIs" dxfId="15" priority="45" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="80" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C53 C56">
-    <cfRule type="cellIs" dxfId="13" priority="43" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="46" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C60:C61">
-    <cfRule type="cellIs" dxfId="11" priority="93" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="95" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="94" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="96" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C63:C64">
-    <cfRule type="cellIs" dxfId="9" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="33" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="34" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C66:C67">
-    <cfRule type="cellIs" dxfId="7" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="29" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="30" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C69:C70">
+    <cfRule type="cellIs" dxfId="7" priority="25" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="26" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C73">
     <cfRule type="cellIs" dxfId="5" priority="23" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1822,19 +1872,19 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C73">
-    <cfRule type="cellIs" dxfId="3" priority="21" operator="equal">
+  <conditionalFormatting sqref="C76">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C76">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="C79">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1843,7 +1893,7 @@
       <formula1>"No, Yes"</formula1>
     </dataValidation>
     <dataValidation showInputMessage="1" showErrorMessage="1" sqref="C9 C12 C61 C64 C67 C70 C15:C28" xr:uid="{87C6F772-FD4B-9449-B9E7-DA0FF0A031BB}"/>
-    <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="C60 C46 C63 C66 C69 C73 C76" xr:uid="{2B929D69-0393-BA4C-AFD3-02F233DB330E}"/>
+    <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="C60 C46 C63 C66 C69 C73 C76 C79" xr:uid="{2B929D69-0393-BA4C-AFD3-02F233DB330E}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1851,6 +1901,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004934E3CB1C58BA43BC6E229E2BF20201" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e33ccc94e63df24f58cb47229b46e190">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87003a75-b64f-4b22-bf19-aa30740e3d46" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f0f7a5bb162b669de9ce8ff8278c29f" ns2:_="">
     <xsd:import namespace="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
@@ -1996,15 +2055,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -2012,6 +2062,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773946F7-566C-458F-95C9-79B0CCE20E87}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2025,14 +2083,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>